<commit_message>
V2 implementation: batch processing, strategies, status tracking
Add batch orchestration with per-customer processing, multi-strategy
search (fullname_ssn, lastname_dob, unique_identifiers), resumable
batches, and status tracking. Includes new ORM models (batch_runs,
customer_status, results, file_status, master_data), FastAPI routers,
Pydantic schemas, and comprehensive test coverage.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/simulated_files/benefits_enrollment.xlsx
+++ b/data/simulated_files/benefits_enrollment.xlsx
@@ -449,10 +449,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>C001</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -481,10 +479,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>C002</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -513,10 +509,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>C003</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -545,10 +539,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>C004</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -577,10 +569,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>C005</t>
-        </is>
+      <c r="A6" t="n">
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -609,10 +599,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>C006</t>
-        </is>
+      <c r="A7" t="n">
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -641,10 +629,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>C007</t>
-        </is>
+      <c r="A8" t="n">
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -673,10 +659,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>C008</t>
-        </is>
+      <c r="A9" t="n">
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -705,10 +689,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>C009</t>
-        </is>
+      <c r="A10" t="n">
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -737,10 +719,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>C010</t>
-        </is>
+      <c r="A11" t="n">
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update regenerated simulated breach files and seed data
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/simulated_files/benefits_enrollment.xlsx
+++ b/data/simulated_files/benefits_enrollment.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benefits Enrollment" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Benefits Enrollment" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>